<commit_message>
EspModule update to ESP32-WROOM-32E-N4, PCB updated and Deliverables generated
</commit_message>
<xml_diff>
--- a/Design-Files/ASCII-v1.2/Deliverables/BOM/ASCII-v1.2.xlsx
+++ b/Design-Files/ASCII-v1.2/Deliverables/BOM/ASCII-v1.2.xlsx
@@ -842,7 +842,7 @@
     <t>6mR</t>
   </si>
   <si>
-    <t>R11, R12, R14, R15, R16, R27, R29</t>
+    <t>R11, R12, R14, R15, R16, R27, R29,R30</t>
   </si>
   <si>
     <t>RES SMD 10K OHM 0.1% 1/16W 0402</t>
@@ -1169,7 +1169,7 @@
     <t>38-SMD Module</t>
   </si>
   <si>
-    <t>ESP32-WROOM-32</t>
+    <t xml:space="preserve">    ESP32-WROOM-32E-N4</t>
   </si>
   <si>
     <t>Crystal</t>
@@ -4051,7 +4051,7 @@
       </c>
       <c r="K54" s="11"/>
     </row>
-    <row r="55" ht="15.75" spans="1:11">
+    <row r="55" spans="1:11">
       <c r="A55" s="2"/>
       <c r="B55" s="7">
         <f>ROW(B55)-ROW($B$2)</f>
@@ -4079,7 +4079,7 @@
         <v>274</v>
       </c>
       <c r="J55" s="9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K55" s="9"/>
     </row>
@@ -4783,7 +4783,7 @@
       </c>
       <c r="K77" s="9"/>
     </row>
-    <row r="78" ht="15.75" spans="1:11">
+    <row r="78" spans="1:11">
       <c r="A78" s="2"/>
       <c r="B78" s="7">
         <f>ROW(B78)-ROW($B$2)</f>

</xml_diff>

<commit_message>
Indctor updated and fresh deliverables generated
</commit_message>
<xml_diff>
--- a/Design-Files/ASCII-v1.2/Deliverables/BOM/ASCII-v1.2.xlsx
+++ b/Design-Files/ASCII-v1.2/Deliverables/BOM/ASCII-v1.2.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="561" uniqueCount="397">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="391">
   <si>
     <t>#</t>
   </si>
@@ -578,28 +578,10 @@
     <t>SM04B-SRSS-TB(LF)(SN)</t>
   </si>
   <si>
-    <t>Inductors</t>
-  </si>
-  <si>
-    <t>L1</t>
-  </si>
-  <si>
-    <t>8.2uH ±20% 7.2A SMD,5.5x5.3mm Power Inductors ROHS</t>
-  </si>
-  <si>
-    <t>YSPIT0550A-8R2M</t>
-  </si>
-  <si>
-    <t>YJYCOIN</t>
-  </si>
-  <si>
-    <t>8.2nH</t>
-  </si>
-  <si>
     <t>Inductor</t>
   </si>
   <si>
-    <t>L2</t>
+    <t>L1,L2</t>
   </si>
   <si>
     <t>5.5A 2.2uH ±20% 7.5A SMD,5.2x5.4x3mm Power Inductors ROHS</t>
@@ -2326,7 +2308,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr codeName="Sheet1"/>
-  <dimension ref="A1:K81"/>
+  <dimension ref="A1:K80"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="15"/>
   <cols>
     <col min="2" max="2" width="3.14285714285714" style="1" customWidth="1"/>
@@ -3507,69 +3489,69 @@
       </c>
       <c r="K37" s="9"/>
     </row>
-    <row r="38" ht="24.75" spans="1:11">
+    <row r="38" ht="36.75" spans="1:11">
       <c r="A38" s="2"/>
       <c r="B38" s="7">
         <f>ROW(B38)-ROW($B$2)</f>
         <v>36</v>
       </c>
-      <c r="C38" s="13" t="s">
+      <c r="C38" s="8" t="s">
         <v>183</v>
       </c>
-      <c r="D38" s="11" t="s">
+      <c r="D38" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="E38" s="12" t="s">
+      <c r="E38" s="10" t="s">
         <v>185</v>
       </c>
-      <c r="F38" s="11" t="s">
+      <c r="F38" s="9" t="s">
         <v>186</v>
       </c>
-      <c r="G38" s="12" t="s">
+      <c r="G38" s="10" t="s">
         <v>186</v>
       </c>
-      <c r="H38" s="11" t="s">
+      <c r="H38" s="9" t="s">
         <v>187</v>
       </c>
-      <c r="I38" s="12" t="s">
+      <c r="I38" s="10" t="s">
         <v>188</v>
       </c>
-      <c r="J38" s="11">
-        <v>1</v>
-      </c>
-      <c r="K38" s="11"/>
-    </row>
-    <row r="39" ht="36.75" spans="1:11">
+      <c r="J38" s="9">
+        <v>2</v>
+      </c>
+      <c r="K38" s="9"/>
+    </row>
+    <row r="39" ht="24.75" spans="1:11">
       <c r="A39" s="2"/>
       <c r="B39" s="7">
         <f>ROW(B39)-ROW($B$2)</f>
         <v>37</v>
       </c>
       <c r="C39" s="8" t="s">
+        <v>183</v>
+      </c>
+      <c r="D39" s="11" t="s">
         <v>189</v>
       </c>
-      <c r="D39" s="9" t="s">
+      <c r="E39" s="12" t="s">
         <v>190</v>
       </c>
-      <c r="E39" s="10" t="s">
+      <c r="F39" s="11" t="s">
         <v>191</v>
       </c>
-      <c r="F39" s="9" t="s">
+      <c r="G39" s="12" t="s">
+        <v>191</v>
+      </c>
+      <c r="H39" s="11" t="s">
         <v>192</v>
       </c>
-      <c r="G39" s="10" t="s">
-        <v>192</v>
-      </c>
-      <c r="H39" s="9" t="s">
+      <c r="I39" s="12" t="s">
         <v>193</v>
       </c>
-      <c r="I39" s="10" t="s">
-        <v>194</v>
-      </c>
-      <c r="J39" s="9">
-        <v>1</v>
-      </c>
-      <c r="K39" s="9"/>
+      <c r="J39" s="11">
+        <v>1</v>
+      </c>
+      <c r="K39" s="11"/>
     </row>
     <row r="40" ht="24.75" spans="1:11">
       <c r="A40" s="2"/>
@@ -3578,62 +3560,62 @@
         <v>38</v>
       </c>
       <c r="C40" s="8" t="s">
-        <v>189</v>
-      </c>
-      <c r="D40" s="11" t="s">
+        <v>183</v>
+      </c>
+      <c r="D40" s="9" t="s">
+        <v>194</v>
+      </c>
+      <c r="E40" s="10" t="s">
         <v>195</v>
       </c>
-      <c r="E40" s="12" t="s">
+      <c r="F40" s="9" t="s">
         <v>196</v>
       </c>
-      <c r="F40" s="11" t="s">
+      <c r="G40" s="10" t="s">
+        <v>196</v>
+      </c>
+      <c r="H40" s="9" t="s">
         <v>197</v>
       </c>
-      <c r="G40" s="12" t="s">
-        <v>197</v>
-      </c>
-      <c r="H40" s="11" t="s">
+      <c r="I40" s="10" t="s">
         <v>198</v>
       </c>
-      <c r="I40" s="12" t="s">
-        <v>199</v>
-      </c>
-      <c r="J40" s="11">
-        <v>1</v>
-      </c>
-      <c r="K40" s="11"/>
-    </row>
-    <row r="41" ht="24.75" spans="1:11">
+      <c r="J40" s="9">
+        <v>1</v>
+      </c>
+      <c r="K40" s="9"/>
+    </row>
+    <row r="41" ht="15.75" spans="1:11">
       <c r="A41" s="2"/>
       <c r="B41" s="7">
         <f>ROW(B41)-ROW($B$2)</f>
         <v>39</v>
       </c>
-      <c r="C41" s="8" t="s">
-        <v>189</v>
-      </c>
-      <c r="D41" s="9" t="s">
+      <c r="C41" s="13" t="s">
+        <v>183</v>
+      </c>
+      <c r="D41" s="11" t="s">
+        <v>199</v>
+      </c>
+      <c r="E41" s="12" t="s">
         <v>200</v>
       </c>
-      <c r="E41" s="10" t="s">
+      <c r="F41" s="11" t="s">
         <v>201</v>
       </c>
-      <c r="F41" s="9" t="s">
+      <c r="G41" s="12" t="s">
         <v>202</v>
       </c>
-      <c r="G41" s="10" t="s">
-        <v>202</v>
-      </c>
-      <c r="H41" s="9" t="s">
+      <c r="H41" s="11" t="s">
+        <v>27</v>
+      </c>
+      <c r="I41" s="12" t="s">
         <v>203</v>
       </c>
-      <c r="I41" s="10" t="s">
-        <v>204</v>
-      </c>
-      <c r="J41" s="9">
-        <v>1</v>
-      </c>
-      <c r="K41" s="9"/>
+      <c r="J41" s="11">
+        <v>1</v>
+      </c>
+      <c r="K41" s="11"/>
     </row>
     <row r="42" ht="15.75" spans="1:11">
       <c r="A42" s="2"/>
@@ -3641,287 +3623,287 @@
         <f>ROW(B42)-ROW($B$2)</f>
         <v>40</v>
       </c>
-      <c r="C42" s="13" t="s">
-        <v>189</v>
-      </c>
-      <c r="D42" s="11" t="s">
+      <c r="C42" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="D42" s="9" t="s">
         <v>205</v>
       </c>
-      <c r="E42" s="12" t="s">
+      <c r="E42" s="10" t="s">
         <v>206</v>
       </c>
-      <c r="F42" s="11" t="s">
+      <c r="F42" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="G42" s="12" t="s">
+      <c r="G42" s="10" t="s">
         <v>208</v>
       </c>
-      <c r="H42" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="I42" s="12" t="s">
+      <c r="H42" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="J42" s="11">
-        <v>1</v>
-      </c>
-      <c r="K42" s="11"/>
-    </row>
-    <row r="43" ht="15.75" spans="1:11">
+      <c r="I42" s="10" t="s">
+        <v>91</v>
+      </c>
+      <c r="J42" s="9">
+        <v>1</v>
+      </c>
+      <c r="K42" s="9"/>
+    </row>
+    <row r="43" ht="48.75" spans="1:11">
       <c r="A43" s="2"/>
       <c r="B43" s="7">
         <f>ROW(B43)-ROW($B$2)</f>
         <v>41</v>
       </c>
       <c r="C43" s="8" t="s">
+        <v>204</v>
+      </c>
+      <c r="D43" s="11" t="s">
         <v>210</v>
       </c>
-      <c r="D43" s="9" t="s">
+      <c r="E43" s="12" t="s">
         <v>211</v>
       </c>
-      <c r="E43" s="10" t="s">
+      <c r="F43" s="11" t="s">
+        <v>207</v>
+      </c>
+      <c r="G43" s="12" t="s">
         <v>212</v>
       </c>
-      <c r="F43" s="9" t="s">
+      <c r="H43" s="11" t="s">
         <v>213</v>
       </c>
-      <c r="G43" s="10" t="s">
-        <v>214</v>
-      </c>
-      <c r="H43" s="9" t="s">
-        <v>215</v>
-      </c>
-      <c r="I43" s="10" t="s">
+      <c r="I43" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="J43" s="9">
-        <v>1</v>
-      </c>
-      <c r="K43" s="9"/>
-    </row>
-    <row r="44" ht="48.75" spans="1:11">
+      <c r="J43" s="11">
+        <v>1</v>
+      </c>
+      <c r="K43" s="11"/>
+    </row>
+    <row r="44" ht="15.75" spans="1:11">
       <c r="A44" s="2"/>
       <c r="B44" s="7">
         <f>ROW(B44)-ROW($B$2)</f>
         <v>42</v>
       </c>
       <c r="C44" s="8" t="s">
-        <v>210</v>
-      </c>
-      <c r="D44" s="11" t="s">
+        <v>214</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="E44" s="10" t="s">
         <v>216</v>
       </c>
-      <c r="E44" s="12" t="s">
+      <c r="F44" s="9" t="s">
         <v>217</v>
       </c>
-      <c r="F44" s="11" t="s">
-        <v>213</v>
-      </c>
-      <c r="G44" s="12" t="s">
+      <c r="G44" s="10" t="s">
         <v>218</v>
       </c>
-      <c r="H44" s="11" t="s">
+      <c r="H44" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I44" s="10" t="s">
         <v>219</v>
       </c>
-      <c r="I44" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="J44" s="11">
-        <v>1</v>
-      </c>
-      <c r="K44" s="11"/>
-    </row>
-    <row r="45" ht="15.75" spans="1:11">
+      <c r="J44" s="9">
+        <v>1</v>
+      </c>
+      <c r="K44" s="9"/>
+    </row>
+    <row r="45" ht="36.75" spans="1:11">
       <c r="A45" s="2"/>
       <c r="B45" s="7">
         <f>ROW(B45)-ROW($B$2)</f>
         <v>43</v>
       </c>
-      <c r="C45" s="8" t="s">
+      <c r="C45" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="D45" s="11" t="s">
         <v>220</v>
       </c>
-      <c r="D45" s="9" t="s">
+      <c r="E45" s="12" t="s">
         <v>221</v>
       </c>
-      <c r="E45" s="10" t="s">
+      <c r="F45" s="11" t="s">
         <v>222</v>
       </c>
-      <c r="F45" s="9" t="s">
+      <c r="G45" s="12" t="s">
         <v>223</v>
       </c>
-      <c r="G45" s="10" t="s">
+      <c r="H45" s="11" t="s">
         <v>224</v>
       </c>
-      <c r="H45" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="I45" s="10" t="s">
+      <c r="I45" s="12" t="s">
         <v>225</v>
       </c>
-      <c r="J45" s="9">
-        <v>1</v>
-      </c>
-      <c r="K45" s="9"/>
-    </row>
-    <row r="46" ht="36.75" spans="1:11">
+      <c r="J45" s="11">
+        <v>1</v>
+      </c>
+      <c r="K45" s="11"/>
+    </row>
+    <row r="46" ht="24.75" spans="1:11">
       <c r="A46" s="2"/>
       <c r="B46" s="7">
         <f>ROW(B46)-ROW($B$2)</f>
         <v>44</v>
       </c>
-      <c r="C46" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="D46" s="11" t="s">
+      <c r="C46" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D46" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="E46" s="12" t="s">
+      <c r="E46" s="10" t="s">
         <v>227</v>
       </c>
-      <c r="F46" s="11" t="s">
+      <c r="F46" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="G46" s="10" t="s">
         <v>228</v>
       </c>
-      <c r="G46" s="12" t="s">
+      <c r="H46" s="9" t="s">
         <v>229</v>
       </c>
-      <c r="H46" s="11" t="s">
+      <c r="I46" s="10" t="s">
         <v>230</v>
       </c>
-      <c r="I46" s="12" t="s">
-        <v>231</v>
-      </c>
-      <c r="J46" s="11">
-        <v>1</v>
-      </c>
-      <c r="K46" s="11"/>
-    </row>
-    <row r="47" ht="24.75" spans="1:11">
+      <c r="J46" s="9">
+        <v>1</v>
+      </c>
+      <c r="K46" s="9"/>
+    </row>
+    <row r="47" ht="36.75" spans="1:11">
       <c r="A47" s="2"/>
       <c r="B47" s="7">
         <f>ROW(B47)-ROW($B$2)</f>
         <v>45</v>
       </c>
-      <c r="C47" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="D47" s="9" t="s">
+      <c r="C47" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="D47" s="11" t="s">
+        <v>231</v>
+      </c>
+      <c r="E47" s="12" t="s">
         <v>232</v>
       </c>
-      <c r="E47" s="10" t="s">
+      <c r="F47" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="G47" s="12" t="s">
         <v>233</v>
       </c>
-      <c r="F47" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="G47" s="10" t="s">
+      <c r="H47" s="11" t="s">
         <v>234</v>
       </c>
-      <c r="H47" s="9" t="s">
+      <c r="I47" s="12" t="s">
         <v>235</v>
       </c>
-      <c r="I47" s="10" t="s">
-        <v>236</v>
-      </c>
-      <c r="J47" s="9">
-        <v>1</v>
-      </c>
-      <c r="K47" s="9"/>
-    </row>
-    <row r="48" ht="36.75" spans="1:11">
+      <c r="J47" s="11">
+        <v>1</v>
+      </c>
+      <c r="K47" s="11"/>
+    </row>
+    <row r="48" ht="15.75" spans="1:11">
       <c r="A48" s="2"/>
       <c r="B48" s="7">
         <f>ROW(B48)-ROW($B$2)</f>
         <v>46</v>
       </c>
-      <c r="C48" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="D48" s="11" t="s">
+      <c r="C48" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D48" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="E48" s="10" t="s">
         <v>237</v>
       </c>
-      <c r="E48" s="12" t="s">
+      <c r="F48" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="G48" s="10" t="s">
         <v>238</v>
       </c>
-      <c r="F48" s="11" t="s">
-        <v>228</v>
-      </c>
-      <c r="G48" s="12" t="s">
+      <c r="H48" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I48" s="10" t="s">
         <v>239</v>
       </c>
-      <c r="H48" s="11" t="s">
-        <v>240</v>
-      </c>
-      <c r="I48" s="12" t="s">
-        <v>241</v>
-      </c>
-      <c r="J48" s="11">
-        <v>1</v>
-      </c>
-      <c r="K48" s="11"/>
-    </row>
-    <row r="49" ht="15.75" spans="1:11">
+      <c r="J48" s="9">
+        <v>1</v>
+      </c>
+      <c r="K48" s="9"/>
+    </row>
+    <row r="49" ht="36.75" spans="1:11">
       <c r="A49" s="2"/>
       <c r="B49" s="7">
         <f>ROW(B49)-ROW($B$2)</f>
         <v>47</v>
       </c>
-      <c r="C49" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="D49" s="9" t="s">
+      <c r="C49" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="D49" s="11" t="s">
+        <v>240</v>
+      </c>
+      <c r="E49" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="F49" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="G49" s="12" t="s">
         <v>242</v>
       </c>
-      <c r="E49" s="10" t="s">
+      <c r="H49" s="11" t="s">
         <v>243</v>
       </c>
-      <c r="F49" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="G49" s="10" t="s">
+      <c r="I49" s="12" t="s">
         <v>244</v>
       </c>
-      <c r="H49" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="I49" s="10" t="s">
-        <v>245</v>
-      </c>
-      <c r="J49" s="9">
-        <v>1</v>
-      </c>
-      <c r="K49" s="9"/>
-    </row>
-    <row r="50" ht="36.75" spans="1:11">
+      <c r="J49" s="11">
+        <v>1</v>
+      </c>
+      <c r="K49" s="11"/>
+    </row>
+    <row r="50" ht="15.75" spans="1:11">
       <c r="A50" s="2"/>
       <c r="B50" s="7">
         <f>ROW(B50)-ROW($B$2)</f>
         <v>48</v>
       </c>
-      <c r="C50" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="D50" s="11" t="s">
+      <c r="C50" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D50" s="9" t="s">
+        <v>245</v>
+      </c>
+      <c r="E50" s="10" t="s">
         <v>246</v>
       </c>
-      <c r="E50" s="12" t="s">
+      <c r="F50" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="G50" s="10" t="s">
         <v>247</v>
       </c>
-      <c r="F50" s="11" t="s">
-        <v>228</v>
-      </c>
-      <c r="G50" s="12" t="s">
+      <c r="H50" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I50" s="10" t="s">
         <v>248</v>
       </c>
-      <c r="H50" s="11" t="s">
-        <v>249</v>
-      </c>
-      <c r="I50" s="12" t="s">
-        <v>250</v>
-      </c>
-      <c r="J50" s="11">
-        <v>1</v>
-      </c>
-      <c r="K50" s="11"/>
+      <c r="J50" s="9">
+        <v>1</v>
+      </c>
+      <c r="K50" s="9"/>
     </row>
     <row r="51" ht="15.75" spans="1:11">
       <c r="A51" s="2"/>
@@ -3929,63 +3911,63 @@
         <f>ROW(B51)-ROW($B$2)</f>
         <v>49</v>
       </c>
-      <c r="C51" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="D51" s="9" t="s">
+      <c r="C51" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="D51" s="11" t="s">
+        <v>249</v>
+      </c>
+      <c r="E51" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="F51" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="G51" s="12" t="s">
         <v>251</v>
       </c>
-      <c r="E51" s="10" t="s">
+      <c r="H51" s="11" t="s">
         <v>252</v>
       </c>
-      <c r="F51" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="G51" s="10" t="s">
+      <c r="I51" s="12" t="s">
         <v>253</v>
       </c>
-      <c r="H51" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="I51" s="10" t="s">
-        <v>254</v>
-      </c>
-      <c r="J51" s="9">
-        <v>1</v>
-      </c>
-      <c r="K51" s="9"/>
-    </row>
-    <row r="52" ht="15.75" spans="1:11">
+      <c r="J51" s="11">
+        <v>1</v>
+      </c>
+      <c r="K51" s="11"/>
+    </row>
+    <row r="52" ht="36.75" spans="1:11">
       <c r="A52" s="2"/>
       <c r="B52" s="7">
         <f>ROW(B52)-ROW($B$2)</f>
         <v>50</v>
       </c>
-      <c r="C52" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="D52" s="11" t="s">
+      <c r="C52" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D52" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="E52" s="10" t="s">
         <v>255</v>
       </c>
-      <c r="E52" s="12" t="s">
+      <c r="F52" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="G52" s="10" t="s">
         <v>256</v>
       </c>
-      <c r="F52" s="11" t="s">
-        <v>228</v>
-      </c>
-      <c r="G52" s="12" t="s">
+      <c r="H52" s="9" t="s">
         <v>257</v>
       </c>
-      <c r="H52" s="11" t="s">
+      <c r="I52" s="10" t="s">
         <v>258</v>
       </c>
-      <c r="I52" s="12" t="s">
-        <v>259</v>
-      </c>
-      <c r="J52" s="11">
-        <v>1</v>
-      </c>
-      <c r="K52" s="11"/>
+      <c r="J52" s="9">
+        <v>2</v>
+      </c>
+      <c r="K52" s="9"/>
     </row>
     <row r="53" ht="36.75" spans="1:11">
       <c r="A53" s="2"/>
@@ -3993,191 +3975,191 @@
         <f>ROW(B53)-ROW($B$2)</f>
         <v>51</v>
       </c>
-      <c r="C53" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="D53" s="9" t="s">
+      <c r="C53" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="D53" s="11" t="s">
+        <v>259</v>
+      </c>
+      <c r="E53" s="12" t="s">
         <v>260</v>
       </c>
-      <c r="E53" s="10" t="s">
+      <c r="F53" s="11" t="s">
         <v>261</v>
       </c>
-      <c r="F53" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="G53" s="10" t="s">
+      <c r="G53" s="12" t="s">
         <v>262</v>
       </c>
-      <c r="H53" s="9" t="s">
+      <c r="H53" s="11" t="s">
         <v>263</v>
       </c>
-      <c r="I53" s="10" t="s">
+      <c r="I53" s="12" t="s">
         <v>264</v>
       </c>
-      <c r="J53" s="9">
-        <v>2</v>
-      </c>
-      <c r="K53" s="9"/>
-    </row>
-    <row r="54" ht="36.75" spans="1:11">
+      <c r="J53" s="11">
+        <v>1</v>
+      </c>
+      <c r="K53" s="11"/>
+    </row>
+    <row r="54" ht="15.75" spans="1:11">
       <c r="A54" s="2"/>
       <c r="B54" s="7">
         <f>ROW(B54)-ROW($B$2)</f>
         <v>52</v>
       </c>
-      <c r="C54" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="D54" s="11" t="s">
+      <c r="C54" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D54" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="E54" s="12" t="s">
+      <c r="E54" s="10" t="s">
         <v>266</v>
       </c>
-      <c r="F54" s="11" t="s">
+      <c r="F54" s="9" t="s">
+        <v>222</v>
+      </c>
+      <c r="G54" s="10" t="s">
         <v>267</v>
       </c>
-      <c r="G54" s="12" t="s">
+      <c r="H54" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I54" s="10" t="s">
         <v>268</v>
       </c>
-      <c r="H54" s="11" t="s">
-        <v>269</v>
-      </c>
-      <c r="I54" s="12" t="s">
-        <v>270</v>
-      </c>
-      <c r="J54" s="11">
-        <v>1</v>
-      </c>
-      <c r="K54" s="11"/>
-    </row>
-    <row r="55" spans="1:11">
+      <c r="J54" s="9">
+        <v>8</v>
+      </c>
+      <c r="K54" s="9"/>
+    </row>
+    <row r="55" ht="24.75" spans="1:11">
       <c r="A55" s="2"/>
       <c r="B55" s="7">
         <f>ROW(B55)-ROW($B$2)</f>
         <v>53</v>
       </c>
-      <c r="C55" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="D55" s="9" t="s">
+      <c r="C55" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="D55" s="11" t="s">
+        <v>269</v>
+      </c>
+      <c r="E55" s="12" t="s">
+        <v>270</v>
+      </c>
+      <c r="F55" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="G55" s="12" t="s">
         <v>271</v>
       </c>
-      <c r="E55" s="10" t="s">
+      <c r="H55" s="11" t="s">
         <v>272</v>
       </c>
-      <c r="F55" s="9" t="s">
-        <v>228</v>
-      </c>
-      <c r="G55" s="10" t="s">
+      <c r="I55" s="12" t="s">
         <v>273</v>
       </c>
-      <c r="H55" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="I55" s="10" t="s">
-        <v>274</v>
-      </c>
-      <c r="J55" s="9">
-        <v>8</v>
-      </c>
-      <c r="K55" s="9"/>
-    </row>
-    <row r="56" ht="24.75" spans="1:11">
+      <c r="J55" s="11">
+        <v>1</v>
+      </c>
+      <c r="K55" s="11"/>
+    </row>
+    <row r="56" ht="15.75" spans="1:11">
       <c r="A56" s="2"/>
       <c r="B56" s="7">
         <f>ROW(B56)-ROW($B$2)</f>
         <v>54</v>
       </c>
-      <c r="C56" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="D56" s="11" t="s">
+      <c r="C56" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D56" s="9" t="s">
+        <v>274</v>
+      </c>
+      <c r="E56" s="10" t="s">
         <v>275</v>
       </c>
-      <c r="E56" s="12" t="s">
+      <c r="F56" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="G56" s="10" t="s">
         <v>276</v>
       </c>
-      <c r="F56" s="11" t="s">
-        <v>228</v>
-      </c>
-      <c r="G56" s="12" t="s">
+      <c r="H56" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I56" s="10" t="s">
         <v>277</v>
       </c>
-      <c r="H56" s="11" t="s">
-        <v>278</v>
-      </c>
-      <c r="I56" s="12" t="s">
-        <v>279</v>
-      </c>
-      <c r="J56" s="11">
-        <v>1</v>
-      </c>
-      <c r="K56" s="11"/>
-    </row>
-    <row r="57" ht="15.75" spans="1:11">
+      <c r="J56" s="9">
+        <v>1</v>
+      </c>
+      <c r="K56" s="9"/>
+    </row>
+    <row r="57" ht="36.75" spans="1:11">
       <c r="A57" s="2"/>
       <c r="B57" s="7">
         <f>ROW(B57)-ROW($B$2)</f>
         <v>55</v>
       </c>
-      <c r="C57" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="D57" s="9" t="s">
+      <c r="C57" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="D57" s="11" t="s">
+        <v>278</v>
+      </c>
+      <c r="E57" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="F57" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="G57" s="12" t="s">
         <v>280</v>
-      </c>
-      <c r="E57" s="10" t="s">
-        <v>281</v>
-      </c>
-      <c r="F57" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="G57" s="10" t="s">
-        <v>282</v>
       </c>
       <c r="H57" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="I57" s="10" t="s">
-        <v>283</v>
-      </c>
-      <c r="J57" s="9">
-        <v>1</v>
-      </c>
-      <c r="K57" s="9"/>
-    </row>
-    <row r="58" ht="36.75" spans="1:11">
+      <c r="I57" s="12" t="s">
+        <v>281</v>
+      </c>
+      <c r="J57" s="11">
+        <v>1</v>
+      </c>
+      <c r="K57" s="11"/>
+    </row>
+    <row r="58" ht="15.75" spans="1:11">
       <c r="A58" s="2"/>
       <c r="B58" s="7">
         <f>ROW(B58)-ROW($B$2)</f>
         <v>56</v>
       </c>
-      <c r="C58" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="D58" s="11" t="s">
+      <c r="C58" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D58" s="9" t="s">
+        <v>282</v>
+      </c>
+      <c r="E58" s="10" t="s">
+        <v>283</v>
+      </c>
+      <c r="F58" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="G58" s="10" t="s">
         <v>284</v>
-      </c>
-      <c r="E58" s="12" t="s">
-        <v>285</v>
-      </c>
-      <c r="F58" s="11" t="s">
-        <v>223</v>
-      </c>
-      <c r="G58" s="12" t="s">
-        <v>286</v>
       </c>
       <c r="H58" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="I58" s="12" t="s">
-        <v>287</v>
-      </c>
-      <c r="J58" s="11">
-        <v>1</v>
-      </c>
-      <c r="K58" s="11"/>
+      <c r="I58" s="10" t="s">
+        <v>285</v>
+      </c>
+      <c r="J58" s="9">
+        <v>1</v>
+      </c>
+      <c r="K58" s="9"/>
     </row>
     <row r="59" ht="15.75" spans="1:11">
       <c r="A59" s="2"/>
@@ -4185,31 +4167,29 @@
         <f>ROW(B59)-ROW($B$2)</f>
         <v>57</v>
       </c>
-      <c r="C59" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="D59" s="9" t="s">
+      <c r="C59" s="13"/>
+      <c r="D59" s="11" t="s">
+        <v>286</v>
+      </c>
+      <c r="E59" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="F59" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="G59" s="12" t="s">
         <v>288</v>
       </c>
-      <c r="E59" s="10" t="s">
+      <c r="H59" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="I59" s="12" t="s">
         <v>289</v>
       </c>
-      <c r="F59" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="G59" s="10" t="s">
-        <v>290</v>
-      </c>
-      <c r="H59" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="I59" s="10" t="s">
-        <v>291</v>
-      </c>
-      <c r="J59" s="9">
-        <v>1</v>
-      </c>
-      <c r="K59" s="9"/>
+      <c r="J59" s="11">
+        <v>1</v>
+      </c>
+      <c r="K59" s="11"/>
     </row>
     <row r="60" ht="15.75" spans="1:11">
       <c r="A60" s="2"/>
@@ -4217,29 +4197,31 @@
         <f>ROW(B60)-ROW($B$2)</f>
         <v>58</v>
       </c>
-      <c r="C60" s="13"/>
-      <c r="D60" s="11" t="s">
+      <c r="C60" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D60" s="9" t="s">
+        <v>290</v>
+      </c>
+      <c r="E60" s="10" t="s">
+        <v>291</v>
+      </c>
+      <c r="F60" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="G60" s="10" t="s">
         <v>292</v>
       </c>
-      <c r="E60" s="12" t="s">
+      <c r="H60" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I60" s="10" t="s">
         <v>293</v>
       </c>
-      <c r="F60" s="11" t="s">
-        <v>228</v>
-      </c>
-      <c r="G60" s="12" t="s">
-        <v>294</v>
-      </c>
-      <c r="H60" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="I60" s="12" t="s">
-        <v>295</v>
-      </c>
-      <c r="J60" s="11">
-        <v>1</v>
-      </c>
-      <c r="K60" s="11"/>
+      <c r="J60" s="9">
+        <v>1</v>
+      </c>
+      <c r="K60" s="9"/>
     </row>
     <row r="61" ht="15.75" spans="1:11">
       <c r="A61" s="2"/>
@@ -4247,31 +4229,31 @@
         <f>ROW(B61)-ROW($B$2)</f>
         <v>59</v>
       </c>
-      <c r="C61" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="D61" s="9" t="s">
+      <c r="C61" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="D61" s="11" t="s">
+        <v>294</v>
+      </c>
+      <c r="E61" s="12" t="s">
+        <v>295</v>
+      </c>
+      <c r="F61" s="11" t="s">
+        <v>222</v>
+      </c>
+      <c r="G61" s="12" t="s">
         <v>296</v>
       </c>
-      <c r="E61" s="10" t="s">
+      <c r="H61" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="I61" s="12" t="s">
         <v>297</v>
       </c>
-      <c r="F61" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="G61" s="10" t="s">
-        <v>298</v>
-      </c>
-      <c r="H61" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="I61" s="10" t="s">
-        <v>299</v>
-      </c>
-      <c r="J61" s="9">
-        <v>1</v>
-      </c>
-      <c r="K61" s="9"/>
+      <c r="J61" s="11">
+        <v>2</v>
+      </c>
+      <c r="K61" s="11"/>
     </row>
     <row r="62" ht="15.75" spans="1:11">
       <c r="A62" s="2"/>
@@ -4279,31 +4261,31 @@
         <f>ROW(B62)-ROW($B$2)</f>
         <v>60</v>
       </c>
-      <c r="C62" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="D62" s="11" t="s">
+      <c r="C62" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D62" s="9" t="s">
+        <v>298</v>
+      </c>
+      <c r="E62" s="10" t="s">
+        <v>299</v>
+      </c>
+      <c r="F62" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="G62" s="10" t="s">
         <v>300</v>
       </c>
-      <c r="E62" s="12" t="s">
+      <c r="H62" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I62" s="10" t="s">
         <v>301</v>
       </c>
-      <c r="F62" s="11" t="s">
-        <v>228</v>
-      </c>
-      <c r="G62" s="12" t="s">
-        <v>302</v>
-      </c>
-      <c r="H62" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="I62" s="12" t="s">
-        <v>303</v>
-      </c>
-      <c r="J62" s="11">
-        <v>2</v>
-      </c>
-      <c r="K62" s="11"/>
+      <c r="J62" s="9">
+        <v>1</v>
+      </c>
+      <c r="K62" s="9"/>
     </row>
     <row r="63" ht="15.75" spans="1:11">
       <c r="A63" s="2"/>
@@ -4311,31 +4293,31 @@
         <f>ROW(B63)-ROW($B$2)</f>
         <v>61</v>
       </c>
-      <c r="C63" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="D63" s="9" t="s">
+      <c r="C63" s="13" t="s">
+        <v>214</v>
+      </c>
+      <c r="D63" s="11" t="s">
+        <v>302</v>
+      </c>
+      <c r="E63" s="12" t="s">
+        <v>303</v>
+      </c>
+      <c r="F63" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="G63" s="12" t="s">
         <v>304</v>
       </c>
-      <c r="E63" s="10" t="s">
+      <c r="H63" s="11" t="s">
+        <v>15</v>
+      </c>
+      <c r="I63" s="12" t="s">
         <v>305</v>
       </c>
-      <c r="F63" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="G63" s="10" t="s">
-        <v>306</v>
-      </c>
-      <c r="H63" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="I63" s="10" t="s">
-        <v>307</v>
-      </c>
-      <c r="J63" s="9">
-        <v>1</v>
-      </c>
-      <c r="K63" s="9"/>
+      <c r="J63" s="11">
+        <v>1</v>
+      </c>
+      <c r="K63" s="11"/>
     </row>
     <row r="64" ht="15.75" spans="1:11">
       <c r="A64" s="2"/>
@@ -4343,31 +4325,31 @@
         <f>ROW(B64)-ROW($B$2)</f>
         <v>62</v>
       </c>
-      <c r="C64" s="13" t="s">
-        <v>220</v>
-      </c>
-      <c r="D64" s="11" t="s">
+      <c r="C64" s="8" t="s">
+        <v>214</v>
+      </c>
+      <c r="D64" s="9" t="s">
+        <v>306</v>
+      </c>
+      <c r="E64" s="10" t="s">
+        <v>307</v>
+      </c>
+      <c r="F64" s="9" t="s">
+        <v>217</v>
+      </c>
+      <c r="G64" s="10" t="s">
         <v>308</v>
       </c>
-      <c r="E64" s="12" t="s">
+      <c r="H64" s="9" t="s">
+        <v>15</v>
+      </c>
+      <c r="I64" s="10" t="s">
         <v>309</v>
       </c>
-      <c r="F64" s="11" t="s">
-        <v>223</v>
-      </c>
-      <c r="G64" s="12" t="s">
-        <v>310</v>
-      </c>
-      <c r="H64" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="I64" s="12" t="s">
-        <v>311</v>
-      </c>
-      <c r="J64" s="11">
-        <v>1</v>
-      </c>
-      <c r="K64" s="11"/>
+      <c r="J64" s="9">
+        <v>1</v>
+      </c>
+      <c r="K64" s="9"/>
     </row>
     <row r="65" ht="15.75" spans="1:11">
       <c r="A65" s="2"/>
@@ -4375,95 +4357,95 @@
         <f>ROW(B65)-ROW($B$2)</f>
         <v>63</v>
       </c>
-      <c r="C65" s="8" t="s">
-        <v>220</v>
-      </c>
-      <c r="D65" s="9" t="s">
+      <c r="C65" s="13" t="s">
+        <v>310</v>
+      </c>
+      <c r="D65" s="11" t="s">
+        <v>311</v>
+      </c>
+      <c r="E65" s="12" t="s">
         <v>312</v>
       </c>
-      <c r="E65" s="10" t="s">
+      <c r="F65" s="11" t="s">
         <v>313</v>
       </c>
-      <c r="F65" s="9" t="s">
-        <v>223</v>
-      </c>
-      <c r="G65" s="10" t="s">
+      <c r="G65" s="12" t="s">
+        <v>313</v>
+      </c>
+      <c r="H65" s="11" t="s">
         <v>314</v>
       </c>
-      <c r="H65" s="9" t="s">
-        <v>15</v>
-      </c>
-      <c r="I65" s="10" t="s">
-        <v>315</v>
-      </c>
-      <c r="J65" s="9">
-        <v>1</v>
-      </c>
-      <c r="K65" s="9"/>
-    </row>
-    <row r="66" ht="15.75" spans="1:11">
+      <c r="I65" s="12" t="s">
+        <v>91</v>
+      </c>
+      <c r="J65" s="11">
+        <v>6</v>
+      </c>
+      <c r="K65" s="11"/>
+    </row>
+    <row r="66" ht="26.25" spans="1:11">
       <c r="A66" s="2"/>
       <c r="B66" s="7">
         <f>ROW(B66)-ROW($B$2)</f>
         <v>64</v>
       </c>
-      <c r="C66" s="13" t="s">
+      <c r="C66" s="8" t="s">
+        <v>315</v>
+      </c>
+      <c r="D66" s="9" t="s">
         <v>316</v>
       </c>
-      <c r="D66" s="11" t="s">
+      <c r="E66" s="10" t="s">
         <v>317</v>
       </c>
-      <c r="E66" s="12" t="s">
+      <c r="F66" s="9" t="s">
         <v>318</v>
       </c>
-      <c r="F66" s="11" t="s">
+      <c r="G66" s="10" t="s">
         <v>319</v>
       </c>
-      <c r="G66" s="12" t="s">
-        <v>319</v>
-      </c>
-      <c r="H66" s="11" t="s">
+      <c r="H66" s="9" t="s">
         <v>320</v>
       </c>
       <c r="I66" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="J66" s="11">
-        <v>6</v>
-      </c>
-      <c r="K66" s="11"/>
-    </row>
-    <row r="67" ht="26.25" spans="1:11">
+      <c r="J66" s="9">
+        <v>3</v>
+      </c>
+      <c r="K66" s="9"/>
+    </row>
+    <row r="67" ht="15.75" spans="1:11">
       <c r="A67" s="2"/>
       <c r="B67" s="7">
         <f>ROW(B67)-ROW($B$2)</f>
         <v>65</v>
       </c>
-      <c r="C67" s="8" t="s">
+      <c r="C67" s="13" t="s">
         <v>321</v>
       </c>
-      <c r="D67" s="9" t="s">
+      <c r="D67" s="11" t="s">
         <v>322</v>
       </c>
-      <c r="E67" s="10" t="s">
+      <c r="E67" s="12" t="s">
         <v>323</v>
       </c>
-      <c r="F67" s="9" t="s">
+      <c r="F67" s="11" t="s">
         <v>324</v>
       </c>
-      <c r="G67" s="10" t="s">
+      <c r="G67" s="12" t="s">
         <v>325</v>
       </c>
-      <c r="H67" s="9" t="s">
+      <c r="H67" s="11" t="s">
         <v>326</v>
       </c>
       <c r="I67" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="J67" s="9">
-        <v>3</v>
-      </c>
-      <c r="K67" s="9"/>
+      <c r="J67" s="11">
+        <v>1</v>
+      </c>
+      <c r="K67" s="11"/>
     </row>
     <row r="68" ht="15.75" spans="1:11">
       <c r="A68" s="2"/>
@@ -4471,95 +4453,95 @@
         <f>ROW(B68)-ROW($B$2)</f>
         <v>66</v>
       </c>
-      <c r="C68" s="13" t="s">
+      <c r="C68" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="D68" s="9" t="s">
         <v>327</v>
       </c>
-      <c r="D68" s="11" t="s">
+      <c r="E68" s="10" t="s">
         <v>328</v>
       </c>
-      <c r="E68" s="12" t="s">
+      <c r="F68" s="9" t="s">
         <v>329</v>
       </c>
-      <c r="F68" s="11" t="s">
+      <c r="G68" s="10" t="s">
         <v>330</v>
       </c>
-      <c r="G68" s="12" t="s">
+      <c r="H68" s="9" t="s">
         <v>331</v>
-      </c>
-      <c r="H68" s="11" t="s">
-        <v>332</v>
       </c>
       <c r="I68" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="J68" s="11">
-        <v>1</v>
-      </c>
-      <c r="K68" s="11"/>
-    </row>
-    <row r="69" ht="15.75" spans="1:11">
+      <c r="J68" s="9">
+        <v>1</v>
+      </c>
+      <c r="K68" s="9"/>
+    </row>
+    <row r="69" ht="36.75" spans="1:11">
       <c r="A69" s="2"/>
       <c r="B69" s="7">
         <f>ROW(B69)-ROW($B$2)</f>
         <v>67</v>
       </c>
       <c r="C69" s="8" t="s">
-        <v>327</v>
-      </c>
-      <c r="D69" s="9" t="s">
+        <v>321</v>
+      </c>
+      <c r="D69" s="11" t="s">
+        <v>332</v>
+      </c>
+      <c r="E69" s="12" t="s">
         <v>333</v>
       </c>
-      <c r="E69" s="10" t="s">
+      <c r="F69" s="11" t="s">
         <v>334</v>
       </c>
-      <c r="F69" s="9" t="s">
+      <c r="G69" s="12" t="s">
         <v>335</v>
       </c>
-      <c r="G69" s="10" t="s">
-        <v>336</v>
-      </c>
-      <c r="H69" s="9" t="s">
-        <v>337</v>
+      <c r="H69" s="11" t="s">
+        <v>91</v>
       </c>
       <c r="I69" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="J69" s="9">
-        <v>1</v>
-      </c>
-      <c r="K69" s="9"/>
-    </row>
-    <row r="70" ht="36.75" spans="1:11">
+      <c r="J69" s="11">
+        <v>1</v>
+      </c>
+      <c r="K69" s="11"/>
+    </row>
+    <row r="70" ht="15.75" spans="1:11">
       <c r="A70" s="2"/>
       <c r="B70" s="7">
         <f>ROW(B70)-ROW($B$2)</f>
         <v>68</v>
       </c>
       <c r="C70" s="8" t="s">
-        <v>327</v>
-      </c>
-      <c r="D70" s="11" t="s">
+        <v>321</v>
+      </c>
+      <c r="D70" s="9" t="s">
+        <v>336</v>
+      </c>
+      <c r="E70" s="10" t="s">
+        <v>337</v>
+      </c>
+      <c r="F70" s="9" t="s">
         <v>338</v>
       </c>
-      <c r="E70" s="12" t="s">
+      <c r="G70" s="10" t="s">
         <v>339</v>
       </c>
-      <c r="F70" s="11" t="s">
+      <c r="H70" s="9" t="s">
         <v>340</v>
-      </c>
-      <c r="G70" s="12" t="s">
-        <v>341</v>
-      </c>
-      <c r="H70" s="11" t="s">
-        <v>91</v>
       </c>
       <c r="I70" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="J70" s="11">
-        <v>1</v>
-      </c>
-      <c r="K70" s="11"/>
+      <c r="J70" s="9">
+        <v>1</v>
+      </c>
+      <c r="K70" s="9"/>
     </row>
     <row r="71" ht="15.75" spans="1:11">
       <c r="A71" s="2"/>
@@ -4567,31 +4549,31 @@
         <f>ROW(B71)-ROW($B$2)</f>
         <v>69</v>
       </c>
-      <c r="C71" s="8" t="s">
-        <v>327</v>
-      </c>
-      <c r="D71" s="9" t="s">
+      <c r="C71" s="13" t="s">
+        <v>321</v>
+      </c>
+      <c r="D71" s="11" t="s">
+        <v>341</v>
+      </c>
+      <c r="E71" s="12" t="s">
         <v>342</v>
       </c>
-      <c r="E71" s="10" t="s">
+      <c r="F71" s="11" t="s">
+        <v>329</v>
+      </c>
+      <c r="G71" s="12" t="s">
         <v>343</v>
       </c>
-      <c r="F71" s="9" t="s">
+      <c r="H71" s="11" t="s">
         <v>344</v>
-      </c>
-      <c r="G71" s="10" t="s">
-        <v>345</v>
-      </c>
-      <c r="H71" s="9" t="s">
-        <v>346</v>
       </c>
       <c r="I71" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="J71" s="9">
-        <v>1</v>
-      </c>
-      <c r="K71" s="9"/>
+      <c r="J71" s="11">
+        <v>1</v>
+      </c>
+      <c r="K71" s="11"/>
     </row>
     <row r="72" ht="15.75" spans="1:11">
       <c r="A72" s="2"/>
@@ -4599,31 +4581,29 @@
         <f>ROW(B72)-ROW($B$2)</f>
         <v>70</v>
       </c>
-      <c r="C72" s="13" t="s">
-        <v>327</v>
-      </c>
-      <c r="D72" s="11" t="s">
+      <c r="C72" s="8"/>
+      <c r="D72" s="9" t="s">
+        <v>345</v>
+      </c>
+      <c r="E72" s="10" t="s">
+        <v>346</v>
+      </c>
+      <c r="F72" s="9" t="s">
         <v>347</v>
       </c>
-      <c r="E72" s="12" t="s">
+      <c r="G72" s="10" t="s">
         <v>348</v>
       </c>
-      <c r="F72" s="11" t="s">
-        <v>335</v>
-      </c>
-      <c r="G72" s="12" t="s">
+      <c r="H72" s="9" t="s">
         <v>349</v>
-      </c>
-      <c r="H72" s="11" t="s">
-        <v>350</v>
       </c>
       <c r="I72" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="J72" s="11">
-        <v>1</v>
-      </c>
-      <c r="K72" s="11"/>
+      <c r="J72" s="9">
+        <v>1</v>
+      </c>
+      <c r="K72" s="9"/>
     </row>
     <row r="73" ht="15.75" spans="1:11">
       <c r="A73" s="2"/>
@@ -4631,29 +4611,31 @@
         <f>ROW(B73)-ROW($B$2)</f>
         <v>71</v>
       </c>
-      <c r="C73" s="8"/>
-      <c r="D73" s="9" t="s">
+      <c r="C73" s="13" t="s">
+        <v>321</v>
+      </c>
+      <c r="D73" s="11" t="s">
+        <v>350</v>
+      </c>
+      <c r="E73" s="12" t="s">
         <v>351</v>
       </c>
-      <c r="E73" s="10" t="s">
+      <c r="F73" s="11" t="s">
         <v>352</v>
       </c>
-      <c r="F73" s="9" t="s">
+      <c r="G73" s="12" t="s">
         <v>353</v>
       </c>
-      <c r="G73" s="10" t="s">
+      <c r="H73" s="11" t="s">
         <v>354</v>
-      </c>
-      <c r="H73" s="9" t="s">
-        <v>355</v>
       </c>
       <c r="I73" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="J73" s="9">
-        <v>1</v>
-      </c>
-      <c r="K73" s="9"/>
+      <c r="J73" s="11">
+        <v>1</v>
+      </c>
+      <c r="K73" s="11"/>
     </row>
     <row r="74" ht="15.75" spans="1:11">
       <c r="A74" s="2"/>
@@ -4661,31 +4643,31 @@
         <f>ROW(B74)-ROW($B$2)</f>
         <v>72</v>
       </c>
-      <c r="C74" s="13" t="s">
-        <v>327</v>
-      </c>
-      <c r="D74" s="11" t="s">
+      <c r="C74" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="D74" s="9" t="s">
+        <v>355</v>
+      </c>
+      <c r="E74" s="10" t="s">
         <v>356</v>
       </c>
-      <c r="E74" s="12" t="s">
+      <c r="F74" s="9" t="s">
         <v>357</v>
       </c>
-      <c r="F74" s="11" t="s">
+      <c r="G74" s="10" t="s">
         <v>358</v>
       </c>
-      <c r="G74" s="12" t="s">
+      <c r="H74" s="9" t="s">
         <v>359</v>
-      </c>
-      <c r="H74" s="11" t="s">
-        <v>360</v>
       </c>
       <c r="I74" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="J74" s="11">
-        <v>1</v>
-      </c>
-      <c r="K74" s="11"/>
+      <c r="J74" s="9">
+        <v>1</v>
+      </c>
+      <c r="K74" s="9"/>
     </row>
     <row r="75" ht="15.75" spans="1:11">
       <c r="A75" s="2"/>
@@ -4693,31 +4675,31 @@
         <f>ROW(B75)-ROW($B$2)</f>
         <v>73</v>
       </c>
-      <c r="C75" s="8" t="s">
-        <v>327</v>
-      </c>
-      <c r="D75" s="9" t="s">
+      <c r="C75" s="13" t="s">
+        <v>321</v>
+      </c>
+      <c r="D75" s="11" t="s">
+        <v>360</v>
+      </c>
+      <c r="E75" s="12" t="s">
         <v>361</v>
       </c>
-      <c r="E75" s="10" t="s">
+      <c r="F75" s="11" t="s">
         <v>362</v>
       </c>
-      <c r="F75" s="9" t="s">
+      <c r="G75" s="12" t="s">
         <v>363</v>
       </c>
-      <c r="G75" s="10" t="s">
+      <c r="H75" s="11" t="s">
         <v>364</v>
-      </c>
-      <c r="H75" s="9" t="s">
-        <v>365</v>
       </c>
       <c r="I75" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="J75" s="9">
-        <v>1</v>
-      </c>
-      <c r="K75" s="9"/>
+      <c r="J75" s="11">
+        <v>1</v>
+      </c>
+      <c r="K75" s="11"/>
     </row>
     <row r="76" ht="15.75" spans="1:11">
       <c r="A76" s="2"/>
@@ -4725,31 +4707,31 @@
         <f>ROW(B76)-ROW($B$2)</f>
         <v>74</v>
       </c>
-      <c r="C76" s="13" t="s">
-        <v>327</v>
-      </c>
-      <c r="D76" s="11" t="s">
+      <c r="C76" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="D76" s="9" t="s">
+        <v>365</v>
+      </c>
+      <c r="E76" s="10" t="s">
         <v>366</v>
       </c>
-      <c r="E76" s="12" t="s">
+      <c r="F76" s="9" t="s">
         <v>367</v>
       </c>
-      <c r="F76" s="11" t="s">
+      <c r="G76" s="10" t="s">
         <v>368</v>
       </c>
-      <c r="G76" s="12" t="s">
+      <c r="H76" s="9" t="s">
         <v>369</v>
-      </c>
-      <c r="H76" s="11" t="s">
-        <v>370</v>
       </c>
       <c r="I76" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="J76" s="11">
-        <v>1</v>
-      </c>
-      <c r="K76" s="11"/>
+      <c r="J76" s="9">
+        <v>1</v>
+      </c>
+      <c r="K76" s="9"/>
     </row>
     <row r="77" ht="15.75" spans="1:11">
       <c r="A77" s="2"/>
@@ -4757,159 +4739,127 @@
         <f>ROW(B77)-ROW($B$2)</f>
         <v>75</v>
       </c>
-      <c r="C77" s="8" t="s">
-        <v>327</v>
-      </c>
-      <c r="D77" s="9" t="s">
+      <c r="C77" s="13" t="s">
+        <v>370</v>
+      </c>
+      <c r="D77" s="11" t="s">
         <v>371</v>
       </c>
-      <c r="E77" s="10" t="s">
+      <c r="E77" s="12" t="s">
         <v>372</v>
       </c>
-      <c r="F77" s="9" t="s">
+      <c r="F77" s="11" t="s">
         <v>373</v>
       </c>
-      <c r="G77" s="10" t="s">
+      <c r="G77" s="12" t="s">
         <v>374</v>
       </c>
-      <c r="H77" s="9" t="s">
-        <v>375</v>
+      <c r="H77" s="11" t="s">
+        <v>326</v>
       </c>
       <c r="I77" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="J77" s="9">
-        <v>1</v>
-      </c>
-      <c r="K77" s="9"/>
-    </row>
-    <row r="78" spans="1:11">
+      <c r="J77" s="11">
+        <v>1</v>
+      </c>
+      <c r="K77" s="11"/>
+    </row>
+    <row r="78" ht="15.75" spans="1:11">
       <c r="A78" s="2"/>
       <c r="B78" s="7">
         <f>ROW(B78)-ROW($B$2)</f>
         <v>76</v>
       </c>
-      <c r="C78" s="13" t="s">
+      <c r="C78" s="8" t="s">
+        <v>375</v>
+      </c>
+      <c r="D78" s="9" t="s">
         <v>376</v>
       </c>
-      <c r="D78" s="11" t="s">
+      <c r="E78" s="10" t="s">
         <v>377</v>
       </c>
-      <c r="E78" s="12" t="s">
+      <c r="F78" s="9" t="s">
         <v>378</v>
       </c>
-      <c r="F78" s="11" t="s">
+      <c r="G78" s="10" t="s">
         <v>379</v>
       </c>
-      <c r="G78" s="12" t="s">
+      <c r="H78" s="9" t="s">
         <v>380</v>
-      </c>
-      <c r="H78" s="11" t="s">
-        <v>332</v>
       </c>
       <c r="I78" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="J78" s="11">
-        <v>1</v>
-      </c>
-      <c r="K78" s="11"/>
-    </row>
-    <row r="79" ht="15.75" spans="1:11">
+      <c r="J78" s="9">
+        <v>1</v>
+      </c>
+      <c r="K78" s="9"/>
+    </row>
+    <row r="79" ht="36.75" spans="1:11">
       <c r="A79" s="2"/>
       <c r="B79" s="7">
         <f>ROW(B79)-ROW($B$2)</f>
         <v>77</v>
       </c>
-      <c r="C79" s="8" t="s">
+      <c r="C79" s="13" t="s">
+        <v>375</v>
+      </c>
+      <c r="D79" s="11" t="s">
         <v>381</v>
       </c>
-      <c r="D79" s="9" t="s">
+      <c r="E79" s="12" t="s">
         <v>382</v>
       </c>
-      <c r="E79" s="10" t="s">
+      <c r="F79" s="11" t="s">
         <v>383</v>
       </c>
-      <c r="F79" s="9" t="s">
+      <c r="G79" s="12" t="s">
         <v>384</v>
       </c>
-      <c r="G79" s="10" t="s">
+      <c r="H79" s="11" t="s">
         <v>385</v>
-      </c>
-      <c r="H79" s="9" t="s">
-        <v>386</v>
       </c>
       <c r="I79" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="J79" s="9">
-        <v>1</v>
-      </c>
-      <c r="K79" s="9"/>
-    </row>
-    <row r="80" ht="36.75" spans="1:11">
+      <c r="J79" s="11">
+        <v>1</v>
+      </c>
+      <c r="K79" s="11"/>
+    </row>
+    <row r="80" ht="15.75" spans="1:11">
       <c r="A80" s="2"/>
       <c r="B80" s="7">
         <f>ROW(B80)-ROW($B$2)</f>
         <v>78</v>
       </c>
       <c r="C80" s="13" t="s">
-        <v>381</v>
-      </c>
-      <c r="D80" s="11" t="s">
+        <v>375</v>
+      </c>
+      <c r="D80" s="9" t="s">
+        <v>386</v>
+      </c>
+      <c r="E80" s="10" t="s">
         <v>387</v>
       </c>
-      <c r="E80" s="12" t="s">
+      <c r="F80" s="9" t="s">
         <v>388</v>
       </c>
-      <c r="F80" s="11" t="s">
+      <c r="G80" s="10" t="s">
         <v>389</v>
       </c>
-      <c r="G80" s="12" t="s">
+      <c r="H80" s="9" t="s">
         <v>390</v>
-      </c>
-      <c r="H80" s="11" t="s">
-        <v>391</v>
       </c>
       <c r="I80" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="J80" s="11">
-        <v>1</v>
-      </c>
-      <c r="K80" s="11"/>
-    </row>
-    <row r="81" ht="15.75" spans="1:11">
-      <c r="A81" s="2"/>
-      <c r="B81" s="7">
-        <f>ROW(B81)-ROW($B$2)</f>
-        <v>79</v>
-      </c>
-      <c r="C81" s="13" t="s">
-        <v>381</v>
-      </c>
-      <c r="D81" s="9" t="s">
-        <v>392</v>
-      </c>
-      <c r="E81" s="10" t="s">
-        <v>393</v>
-      </c>
-      <c r="F81" s="9" t="s">
-        <v>394</v>
-      </c>
-      <c r="G81" s="10" t="s">
-        <v>395</v>
-      </c>
-      <c r="H81" s="9" t="s">
-        <v>396</v>
-      </c>
-      <c r="I81" s="12" t="s">
-        <v>91</v>
-      </c>
-      <c r="J81" s="9">
-        <v>1</v>
-      </c>
-      <c r="K81" s="9"/>
+      <c r="J80" s="9">
+        <v>1</v>
+      </c>
+      <c r="K80" s="9"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>

<commit_message>
R18 updated with new part num RC0603FR-0715K4L, BOM and schematic updated acc:
</commit_message>
<xml_diff>
--- a/Design-Files/ASCII-v1.2/Deliverables/BOM/ASCII-v1.2.xlsx
+++ b/Design-Files/ASCII-v1.2/Deliverables/BOM/ASCII-v1.2.xlsx
@@ -866,10 +866,10 @@
     <t>R18</t>
   </si>
   <si>
-    <t>SMD Chip Resistor, 15.4 kOhm, ± 1%, 50 mW, 0201 [0603 Metric], Thick Film, General Purpose</t>
-  </si>
-  <si>
-    <t>RC0201FR-0715K4L</t>
+    <t>100mW Thick Film Resistors 75V ±100ppm/℃ ±1% 15.4kΩ 0603 Chip Resistor - Surface Mount ROHS</t>
+  </si>
+  <si>
+    <t>RC0603FR-0715K4L</t>
   </si>
   <si>
     <t>15.4K</t>

</xml_diff>